<commit_message>
Fix Google Sheets updates without rewriting existing rows
</commit_message>
<xml_diff>
--- a/results/DailyStats.xlsx
+++ b/results/DailyStats.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R76"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4044,6 +4044,102 @@
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr"/>
     </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>20260905</v>
+      </c>
+      <c r="B77" t="n">
+        <v>170</v>
+      </c>
+      <c r="C77" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="D77" t="n">
+        <v>164.42</v>
+      </c>
+      <c r="E77" t="n">
+        <v>930</v>
+      </c>
+      <c r="F77" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="G77" t="n">
+        <v>899.9</v>
+      </c>
+      <c r="H77" t="n">
+        <v>2</v>
+      </c>
+      <c r="I77" t="n">
+        <v>7</v>
+      </c>
+      <c r="J77" t="n">
+        <v>6</v>
+      </c>
+      <c r="K77" t="n">
+        <v>4</v>
+      </c>
+      <c r="L77" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" t="n">
+        <v>1</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0</v>
+      </c>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>20260911</v>
+      </c>
+      <c r="B78" t="n">
+        <v>50</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D78" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="E78" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F78" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1952.2</v>
+      </c>
+      <c r="H78" t="n">
+        <v>2</v>
+      </c>
+      <c r="I78" t="n">
+        <v>2</v>
+      </c>
+      <c r="J78" t="n">
+        <v>4</v>
+      </c>
+      <c r="K78" t="n">
+        <v>2</v>
+      </c>
+      <c r="L78" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" t="n">
+        <v>1</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>